<commit_message>
Update generated matching outputs
</commit_message>
<xml_diff>
--- a/generated/committee_recommendations.xlsx
+++ b/generated/committee_recommendations.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,65 +473,901 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>佐藤健</t>
+          <t>但木 陸</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>都市交通需要予測に対する時系列深層学習の適用</t>
+          <t>大学入試業務の人員配置最適化における数理モデルの改良</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>鈴木花子</t>
+          <t>高野祐一</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>山田太郎</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
+          <t>繁野麻衣子</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>吉瀬章子</t>
+        </is>
+      </c>
       <c r="F2" t="n">
-        <v>0.442595083489533</v>
+        <v>0.7990804751472282</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2112356007377654</v>
+        <v>0.7457407141319889</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>0.7436180316601839</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>田中葵</t>
+          <t>吉田 響</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>災害時避難行動データを用いた最適配置モデルの研究</t>
+          <t>社会工学・サービス工学学位プログラムにおける修士論文審査員の割り当て問題</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>鈴木花子</t>
+          <t>原田信行</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>山田太郎</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+          <t>繁野麻衣子</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>秋山英三</t>
+        </is>
+      </c>
       <c r="F3" t="n">
-        <v>0.579686085202809</v>
+        <v>0.7645546623853985</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2974948991787114</v>
+        <v>0.7560855235494532</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>0.7519666255181408</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>金原 壮汰</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>LiDARデータに基づく視線および姿勢情報統合による危険行動の動的検出システム〜荷役作業ケース</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>黒瀬雄大</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>木下陽平</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>岡田幸彦</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0.7730844708148208</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.7492663532653359</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.7377681360832717</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>宍戸 唯輝</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3階層サプライチェーンにおける協調的納期決定アルゴリズム</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>LiuTianxiang</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Phung-DucTuan</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>高野祐一</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>0.7807969700848041</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.7802955162809034</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.7629236394713367</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>堤 敬信</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>閉鎖型待ち行列ネットワークモデルを用いたシェアサイクルの運用分析</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>秋山英三</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>TranLamAnhDuong</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>佐野幸恵</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>0.777475428793001</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.7589512752102814</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.7599317009143467</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>寺田 海渡</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>中小企業デフォルト予測における月次流動性預金残高特徴量の有効性検証</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>大久保正勝</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>TranLamAnhDuong</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>原田信行</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>0.793365402119634</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.7704139251473998</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.7705694203287918</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>益子 颯太</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>仕訳データの異常検知モデルの高度化：Data Collaboration解析と摘要欄の活用</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>黒瀬雄大</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>岡田幸彦</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>吉瀬章子</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>0.7940385736544479</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.7610796693064201</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.75741082965535</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>平井 佑樹</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>仕訳データを用いた利速測定の研究</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>大西正輝</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>黒瀬雄大</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>小西葉子</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>0.7926388773523594</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.7877466609819869</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.7493271465883786</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>飯田 真実</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HPVワクチン接種に対する意見の変遷とその要因</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>大西正輝</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>LiuTianxiang</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>佐野幸恵</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>0.7691184801505473</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.7682644978240212</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.7133311424561222</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>川井 貫太朗</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SNSを用いた労働者の集団感情分析</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>佐野幸恵</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>TranLamAnhDuong</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>秋山英三</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>0.7986562750682954</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.7927969203779757</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.7810778899836618</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>冨樫 歩大</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>テキスト情報と財務情報の統合による中小企業の将来性予測</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>原田信行</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>TranLamAnhDuong</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>岡田幸彦</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>0.7900498149708934</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.7786515345644294</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.725379641877675</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>出口 達也</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>地域要因を用いた慢性腎臓病患者の悪化予測の研究</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TranLamAnhDuong</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>大久保正勝</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>岡田幸彦</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>0.8140611779324148</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.7479848455984035</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.7371903975067992</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>長谷川 弘貴</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>生体情報とテンソルデータ解析によるコンサート満足度の研究</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>岡本直久</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>黒瀬雄大</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>讃井知</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>0.7821082462268162</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.7676686179623895</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.7572288631246638</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>中山 友琉</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>特異値分解を用いた効率的な分散データファインチューニング手法の提案</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>黒瀬雄大</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>繁野麻衣子</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>高野祐一</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>0.7824792788319687</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.7662843099258541</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.7643935545360966</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>齋藤 彩</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>地域愛着の規定因に関する実証分析：つながりの影響の検討</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>讃井知</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>岡本直久</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>小西葉子</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>0.7914804368112953</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.7809460412806564</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.7260086165237314</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>李 宗晟</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>エラスティック光ネットワークにおける通信要求の保持時間を考慮した予約種別リソース割り当て戦略の提案</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Phung-DucTuan</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>LiuTianxiang</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>張勇兵</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>0.7838991994343767</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.7700758577991739</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.7349688599838846</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>澤口 瑛都</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>列生成法を軸とした電気バスの仕業編成最適化</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>高野祐一</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>繁野麻衣子</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>吉瀬章子</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>0.8087958270757369</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.7325343050318592</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.7298264185003422</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>中本 武志</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>大規模言語モデルを活用した非専門家による継続運用可能な勤務表作成手法の検討</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Phung-DucTuan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>黒瀬雄大</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>有馬澄佳</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>0.8145593294894845</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.6931889628284444</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.6843139670630791</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>髙橋 優介</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>重量・近接規制を考慮した異種ドローン経路問題：規制による配送時間・コストへの影響分析</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>高野祐一</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>秋山英三</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>髙橋裕紀</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0.7922602110802039</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.7447926232143768</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.7327941651160159</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>鈴木 颯斗</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>最適多分木を用いた解釈可能なクラスタリング</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>高野祐一</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>吉瀬章子</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>八森正泰</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>0.8031707666476058</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.7521326585034569</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.7488486792745004</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>佐川 翼</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>社会工学・サービス工学学位プログラムにおける修士論文発表会スケジューリングシステムの開発</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>佐野幸恵</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>秋山英三</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>繁野麻衣子</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0.7747239808897584</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.7675358273173142</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.750361214367077</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>加田 昌杜</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>学年暦の自動生成 〜曜日変更最小化モデルとその修正の自動化〜</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>高野祐一</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>繁野麻衣子</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>吉瀬章子</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0.7861770081289896</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.7544270065638702</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.7540988778190654</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>八角 朋樹</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>機械学習モデルと特徴量選択によるファミリーレストラン店舗別売上予測方法の検討</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>高野祐一</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>繁野麻衣子</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>小西葉子</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>0.783767485062085</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.7504054209416953</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.7363430054106848</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>山下 穂乃花</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Continual Learning by Null Space of Weight Matrix of Previous Task for Deep Neural Network</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>繁野麻衣子</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>張勇兵</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>八森正泰</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>0.8210970053065357</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.7549542035323578</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.75543937381531</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>崔 涵喬</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>観光客のセグメンテーションとマーケティングへの応用可能性に関する研究</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>岡本直久</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>秋山英三</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>小西葉子</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>0.814169194661074</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.7201431580307053</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.7087410383921012</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Apply modified matching changes
</commit_message>
<xml_diff>
--- a/generated/committee_recommendations.xlsx
+++ b/generated/committee_recommendations.xlsx
@@ -497,13 +497,13 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.7980324189169082</v>
+        <v>0.7990804751472282</v>
       </c>
       <c r="G2" t="n">
-        <v>0.7476459495927925</v>
+        <v>0.7457407141319889</v>
       </c>
       <c r="H2" t="n">
-        <v>0.745967923074087</v>
+        <v>0.7436180316601839</v>
       </c>
     </row>
     <row r="3">
@@ -533,13 +533,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.7646012657634985</v>
+        <v>0.7645546623853985</v>
       </c>
       <c r="G3" t="n">
-        <v>0.7542134458195275</v>
+        <v>0.7560855235494532</v>
       </c>
       <c r="H3" t="n">
-        <v>0.7485639766309413</v>
+        <v>0.7519666255181408</v>
       </c>
     </row>
     <row r="4">
@@ -569,13 +569,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.7730491480516837</v>
+        <v>0.7730844708148208</v>
       </c>
       <c r="G4" t="n">
-        <v>0.749730500747122</v>
+        <v>0.7492663532653359</v>
       </c>
       <c r="H4" t="n">
-        <v>0.7382624589564942</v>
+        <v>0.7377681360832717</v>
       </c>
     </row>
     <row r="5">
@@ -591,27 +591,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Phung DucTuan</t>
+          <t>LiuTianxiang</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>Phung-DucTuan</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>高野祐一</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>有馬澄佳</t>
-        </is>
-      </c>
       <c r="F5" t="n">
-        <v>0.7948736779933087</v>
+        <v>0.7807969700848041</v>
       </c>
       <c r="G5" t="n">
-        <v>0.7307908669503085</v>
+        <v>0.7802955162809034</v>
       </c>
       <c r="H5" t="n">
-        <v>0.7273656892848034</v>
+        <v>0.7629236394713367</v>
       </c>
     </row>
     <row r="6">
@@ -627,27 +627,27 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Phung DucTuan</t>
+          <t>秋山英三</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>秋山英三</t>
+          <t>TranLamAnhDuong</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Tran Lam Anh Duong</t>
+          <t>佐野幸恵</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.7806034182445172</v>
+        <v>0.777475428793001</v>
       </c>
       <c r="G6" t="n">
-        <v>0.7666447199205355</v>
+        <v>0.7589512752102814</v>
       </c>
       <c r="H6" t="n">
-        <v>0.7472143551988655</v>
+        <v>0.7599317009143467</v>
       </c>
     </row>
     <row r="7">
@@ -668,22 +668,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>TranLamAnhDuong</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>原田信行</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>黒瀬雄大</t>
-        </is>
-      </c>
       <c r="F7" t="n">
-        <v>0.7934823490723095</v>
+        <v>0.793365402119634</v>
       </c>
       <c r="G7" t="n">
-        <v>0.7708026639766218</v>
+        <v>0.7704139251473998</v>
       </c>
       <c r="H7" t="n">
-        <v>0.747030667028405</v>
+        <v>0.7705694203287918</v>
       </c>
     </row>
     <row r="8">
@@ -713,13 +713,13 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.7937366282266973</v>
+        <v>0.7940385736544479</v>
       </c>
       <c r="G8" t="n">
-        <v>0.7604838642054538</v>
+        <v>0.7610796693064201</v>
       </c>
       <c r="H8" t="n">
-        <v>0.7573704867578485</v>
+        <v>0.75741082965535</v>
       </c>
     </row>
     <row r="9">
@@ -749,13 +749,13 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.7916116180778753</v>
+        <v>0.7926388773523594</v>
       </c>
       <c r="G9" t="n">
-        <v>0.7898925298906265</v>
+        <v>0.7877466609819869</v>
       </c>
       <c r="H9" t="n">
-        <v>0.7455020044017525</v>
+        <v>0.7493271465883786</v>
       </c>
     </row>
     <row r="10">
@@ -776,7 +776,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Phung DucTuan</t>
+          <t>LiuTianxiang</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -785,13 +785,13 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.7715006839331053</v>
+        <v>0.7691184801505473</v>
       </c>
       <c r="G10" t="n">
-        <v>0.7343256014576269</v>
+        <v>0.7682644978240212</v>
       </c>
       <c r="H10" t="n">
-        <v>0.7080079314742604</v>
+        <v>0.7133311424561222</v>
       </c>
     </row>
     <row r="11">
@@ -812,22 +812,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>TranLamAnhDuong</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>秋山英三</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>作道真理</t>
-        </is>
-      </c>
       <c r="F11" t="n">
-        <v>0.7987352560391006</v>
+        <v>0.7986562750682954</v>
       </c>
       <c r="G11" t="n">
-        <v>0.780725968062059</v>
+        <v>0.7927969203779757</v>
       </c>
       <c r="H11" t="n">
-        <v>0.7535015021715852</v>
+        <v>0.7810778899836618</v>
       </c>
     </row>
     <row r="12">
@@ -848,7 +848,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Phung DucTuan</t>
+          <t>TranLamAnhDuong</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -857,13 +857,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.790145127807668</v>
+        <v>0.7900498149708934</v>
       </c>
       <c r="G12" t="n">
-        <v>0.7164647088437599</v>
+        <v>0.7786515345644294</v>
       </c>
       <c r="H12" t="n">
-        <v>0.7259820112678075</v>
+        <v>0.725379641877675</v>
       </c>
     </row>
     <row r="13">
@@ -879,7 +879,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Phung DucTuan</t>
+          <t>TranLamAnhDuong</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -893,13 +893,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.8039493044152165</v>
+        <v>0.8140611779324148</v>
       </c>
       <c r="G13" t="n">
-        <v>0.7679389095274342</v>
+        <v>0.7479848455984035</v>
       </c>
       <c r="H13" t="n">
-        <v>0.7559164131217846</v>
+        <v>0.7371903975067992</v>
       </c>
     </row>
     <row r="14">
@@ -929,13 +929,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.7820176892100249</v>
+        <v>0.7821082462268162</v>
       </c>
       <c r="G14" t="n">
-        <v>0.766323994656363</v>
+        <v>0.7676686179623895</v>
       </c>
       <c r="H14" t="n">
-        <v>0.7547788508099192</v>
+        <v>0.7572288631246638</v>
       </c>
     </row>
     <row r="15">
@@ -965,13 +965,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.7822583937871146</v>
+        <v>0.7824792788319687</v>
       </c>
       <c r="G15" t="n">
-        <v>0.7670135299720341</v>
+        <v>0.7662843099258541</v>
       </c>
       <c r="H15" t="n">
-        <v>0.7624678544637103</v>
+        <v>0.7643935545360966</v>
       </c>
     </row>
     <row r="16">
@@ -1001,13 +1001,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.7913745143188848</v>
+        <v>0.7914804368112953</v>
       </c>
       <c r="G16" t="n">
-        <v>0.7797478985608814</v>
+        <v>0.7809460412806564</v>
       </c>
       <c r="H16" t="n">
-        <v>0.721518415283814</v>
+        <v>0.7260086165237314</v>
       </c>
     </row>
     <row r="17">
@@ -1023,27 +1023,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Phung DucTuan</t>
+          <t>Phung-DucTuan</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
+          <t>LiuTianxiang</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>張勇兵</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>高野祐一</t>
-        </is>
-      </c>
       <c r="F17" t="n">
-        <v>0.8022595901834515</v>
+        <v>0.7838991994343767</v>
       </c>
       <c r="G17" t="n">
-        <v>0.7080182967337185</v>
+        <v>0.7700758577991739</v>
       </c>
       <c r="H17" t="n">
-        <v>0.6946508938559388</v>
+        <v>0.7349688599838846</v>
       </c>
     </row>
     <row r="18">
@@ -1069,17 +1069,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Phung DucTuan</t>
+          <t>吉瀬章子</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.8074081286133804</v>
+        <v>0.8087958270757369</v>
       </c>
       <c r="G18" t="n">
-        <v>0.7342494314362839</v>
+        <v>0.7325343050318592</v>
       </c>
       <c r="H18" t="n">
-        <v>0.7239668004375618</v>
+        <v>0.7298264185003422</v>
       </c>
     </row>
     <row r="19">
@@ -1095,27 +1095,27 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>Phung-DucTuan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
           <t>黒瀬雄大</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>有馬澄佳</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>大久保正勝</t>
-        </is>
-      </c>
       <c r="F19" t="n">
-        <v>0.7710509269969877</v>
+        <v>0.8145593294894845</v>
       </c>
       <c r="G19" t="n">
-        <v>0.7593669993368094</v>
+        <v>0.6931889628284444</v>
       </c>
       <c r="H19" t="n">
-        <v>0.743980413093444</v>
+        <v>0.6843139670630791</v>
       </c>
     </row>
     <row r="20">
@@ -1136,22 +1136,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Tran Lam Anh Duong</t>
+          <t>秋山英三</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>秋山英三</t>
+          <t>髙橋裕紀</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.7917937472707031</v>
+        <v>0.7922602110802039</v>
       </c>
       <c r="G20" t="n">
-        <v>0.7576218148018588</v>
+        <v>0.7447926232143768</v>
       </c>
       <c r="H20" t="n">
-        <v>0.7455660530617956</v>
+        <v>0.7327941651160159</v>
       </c>
     </row>
     <row r="21">
@@ -1172,22 +1172,22 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Liu Tianxiang</t>
+          <t>吉瀬章子</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>吉瀬章子</t>
+          <t>八森正泰</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.8020794856104024</v>
+        <v>0.8031707666476058</v>
       </c>
       <c r="G21" t="n">
-        <v>0.7792631197856266</v>
+        <v>0.7521326585034569</v>
       </c>
       <c r="H21" t="n">
-        <v>0.7548336135955751</v>
+        <v>0.7488486792745004</v>
       </c>
     </row>
     <row r="22">
@@ -1213,17 +1213,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Phung DucTuan</t>
+          <t>繁野麻衣子</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.7748048081702387</v>
+        <v>0.7747239808897584</v>
       </c>
       <c r="G22" t="n">
-        <v>0.7662738286239533</v>
+        <v>0.7675358273173142</v>
       </c>
       <c r="H22" t="n">
-        <v>0.7395404025384898</v>
+        <v>0.750361214367077</v>
       </c>
     </row>
     <row r="23">
@@ -1244,22 +1244,22 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Liu Tianxiang</t>
+          <t>繁野麻衣子</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>繁野麻衣子</t>
+          <t>吉瀬章子</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.7852747180597276</v>
+        <v>0.7861770081289896</v>
       </c>
       <c r="G23" t="n">
-        <v>0.76053871506522</v>
+        <v>0.7544270065638702</v>
       </c>
       <c r="H23" t="n">
-        <v>0.7564891461325435</v>
+        <v>0.7540988778190654</v>
       </c>
     </row>
     <row r="24">
@@ -1280,22 +1280,22 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Phung DucTuan</t>
+          <t>繁野麻衣子</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>繁野麻衣子</t>
+          <t>小西葉子</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.7832724380676721</v>
+        <v>0.783767485062085</v>
       </c>
       <c r="G24" t="n">
-        <v>0.751198502802636</v>
+        <v>0.7504054209416953</v>
       </c>
       <c r="H24" t="n">
-        <v>0.7517470788490264</v>
+        <v>0.7363430054106848</v>
       </c>
     </row>
     <row r="25">
@@ -1316,22 +1316,22 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Liu Tianxiang</t>
+          <t>張勇兵</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>張勇兵</t>
+          <t>八森正泰</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>0.8202514556630865</v>
+        <v>0.8210970053065357</v>
       </c>
       <c r="G25" t="n">
-        <v>0.7815374074296739</v>
+        <v>0.7549542035323578</v>
       </c>
       <c r="H25" t="n">
-        <v>0.7536571363979294</v>
+        <v>0.75543937381531</v>
       </c>
     </row>
     <row r="26">
@@ -1361,13 +1361,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0.814105680937531</v>
+        <v>0.814169194661074</v>
       </c>
       <c r="G26" t="n">
-        <v>0.7197502719371935</v>
+        <v>0.7201431580307053</v>
       </c>
       <c r="H26" t="n">
-        <v>0.7064874531815901</v>
+        <v>0.7087410383921012</v>
       </c>
     </row>
   </sheetData>

</xml_diff>